<commit_message>
added per board quantity in PCBWay BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/PCBWay_BOM.xlsx
+++ b/Deliverables/BOM/PCBWay_BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25726"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\JohnWollam-LCDProject\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\JohnWollam-LCDProject\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C4283D2-F5CD-46E9-A4C2-92E47DEC178C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -626,9 +625,6 @@
     <t>8MHZ</t>
   </si>
   <si>
-    <t xml:space="preserve"> Quantity (25 Boards)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> MOQ (25 Boards)</t>
   </si>
   <si>
@@ -657,12 +653,15 @@
   </si>
   <si>
     <t>5TJ480000XYLBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Quantity per board</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1421,7 +1420,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09969436-8A94-45CE-BB95-34EF24CD6072}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{09969436-8A94-45CE-BB95-34EF24CD6072}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1717,7 +1716,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1746,7 +1745,7 @@
       </c>
       <c r="E2" s="36"/>
       <c r="F2" s="69" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G2" s="9"/>
       <c r="H2" s="2"/>
@@ -1764,7 +1763,7 @@
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="70" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="3"/>
@@ -1782,7 +1781,7 @@
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="71" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="5"/>
@@ -1881,10 +1880,10 @@
         <v>154</v>
       </c>
       <c r="K9" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="L9" s="23" t="s">
         <v>198</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>199</v>
       </c>
       <c r="M9" s="23" t="s">
         <v>37</v>
@@ -1920,7 +1919,7 @@
         <v>29</v>
       </c>
       <c r="K10" s="48">
-        <v>150</v>
+        <v>6</v>
       </c>
       <c r="L10" s="48">
         <v>200</v>
@@ -1957,7 +1956,7 @@
         <v>30</v>
       </c>
       <c r="K11" s="50">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="L11" s="50">
         <v>100</v>
@@ -1994,7 +1993,7 @@
         <v>32</v>
       </c>
       <c r="K12" s="52">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="L12" s="52">
         <v>60</v>
@@ -2031,7 +2030,7 @@
         <v>159</v>
       </c>
       <c r="K13" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L13" s="50">
         <v>100</v>
@@ -2068,7 +2067,7 @@
         <v>31</v>
       </c>
       <c r="K14" s="52">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="L14" s="52">
         <v>60</v>
@@ -2105,7 +2104,7 @@
         <v>162</v>
       </c>
       <c r="K15" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L15" s="50">
         <v>100</v>
@@ -2142,7 +2141,7 @@
         <v>164</v>
       </c>
       <c r="K16" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L16" s="52">
         <v>28</v>
@@ -2179,7 +2178,7 @@
         <v>166</v>
       </c>
       <c r="K17" s="55">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L17" s="55">
         <v>28</v>
@@ -2216,7 +2215,7 @@
         <v>144</v>
       </c>
       <c r="K18" s="52">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="L18" s="52">
         <v>60</v>
@@ -2253,7 +2252,7 @@
         <v>144</v>
       </c>
       <c r="K19" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L19" s="50">
         <v>40</v>
@@ -2278,7 +2277,7 @@
         <v>34</v>
       </c>
       <c r="G20" s="62" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H20" s="52" t="s">
         <v>127</v>
@@ -2290,7 +2289,7 @@
         <v>144</v>
       </c>
       <c r="K20" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L20" s="52">
         <v>28</v>
@@ -2327,7 +2326,7 @@
         <v>144</v>
       </c>
       <c r="K21" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L21" s="50">
         <v>30</v>
@@ -2352,7 +2351,7 @@
         <v>34</v>
       </c>
       <c r="G22" s="73" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H22" s="52" t="s">
         <v>130</v>
@@ -2364,7 +2363,7 @@
         <v>144</v>
       </c>
       <c r="K22" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L22" s="52">
         <v>30</v>
@@ -2401,7 +2400,7 @@
         <v>173</v>
       </c>
       <c r="K23" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L23" s="50">
         <v>28</v>
@@ -2426,7 +2425,7 @@
         <v>34</v>
       </c>
       <c r="G24" s="62" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H24" s="52" t="s">
         <v>35</v>
@@ -2438,7 +2437,7 @@
         <v>144</v>
       </c>
       <c r="K24" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L24" s="52">
         <v>50</v>
@@ -2463,7 +2462,7 @@
         <v>21</v>
       </c>
       <c r="G25" s="74" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H25" s="50" t="s">
         <v>133</v>
@@ -2475,7 +2474,7 @@
         <v>144</v>
       </c>
       <c r="K25" s="50">
-        <v>150</v>
+        <v>6</v>
       </c>
       <c r="L25" s="50">
         <v>160</v>
@@ -2500,7 +2499,7 @@
         <v>80</v>
       </c>
       <c r="G26" s="65" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H26" s="52" t="s">
         <v>134</v>
@@ -2512,7 +2511,7 @@
         <v>177</v>
       </c>
       <c r="K26" s="52">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="L26" s="52">
         <v>60</v>
@@ -2537,7 +2536,7 @@
         <v>83</v>
       </c>
       <c r="G27" s="74" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H27" s="50" t="s">
         <v>135</v>
@@ -2549,7 +2548,7 @@
         <v>179</v>
       </c>
       <c r="K27" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L27" s="50">
         <v>50</v>
@@ -2586,7 +2585,7 @@
         <v>181</v>
       </c>
       <c r="K28" s="52">
-        <v>275</v>
+        <v>11</v>
       </c>
       <c r="L28" s="52">
         <v>300</v>
@@ -2623,7 +2622,7 @@
         <v>33</v>
       </c>
       <c r="K29" s="50">
-        <v>325</v>
+        <v>13</v>
       </c>
       <c r="L29" s="50">
         <v>400</v>
@@ -2660,7 +2659,7 @@
         <v>184</v>
       </c>
       <c r="K30" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L30" s="52">
         <v>100</v>
@@ -2697,7 +2696,7 @@
         <v>186</v>
       </c>
       <c r="K31" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L31" s="50">
         <v>50</v>
@@ -2734,7 +2733,7 @@
         <v>188</v>
       </c>
       <c r="K32" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L32" s="52">
         <v>28</v>
@@ -2771,7 +2770,7 @@
         <v>190</v>
       </c>
       <c r="K33" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L33" s="50">
         <v>100</v>
@@ -2808,7 +2807,7 @@
         <v>144</v>
       </c>
       <c r="K34" s="57">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L34" s="57" t="s">
         <v>144</v>
@@ -2845,7 +2844,7 @@
         <v>144</v>
       </c>
       <c r="K35" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L35" s="50">
         <v>28</v>
@@ -2882,7 +2881,7 @@
         <v>144</v>
       </c>
       <c r="K36" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L36" s="52">
         <v>27</v>
@@ -2919,7 +2918,7 @@
         <v>144</v>
       </c>
       <c r="K37" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L37" s="50">
         <v>27</v>
@@ -2956,7 +2955,7 @@
         <v>144</v>
       </c>
       <c r="K38" s="52">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L38" s="52">
         <v>27</v>
@@ -2993,7 +2992,7 @@
         <v>144</v>
       </c>
       <c r="K39" s="50">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L39" s="50">
         <v>30</v>
@@ -3018,7 +3017,7 @@
         <v>34</v>
       </c>
       <c r="G40" s="52" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H40" s="59" t="s">
         <v>152</v>
@@ -3030,7 +3029,7 @@
         <v>197</v>
       </c>
       <c r="K40" s="59">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L40" s="59">
         <v>30</v>

</xml_diff>